<commit_message>
feat(pms): completato Step 21 - integrato SourceQueryFormatter nell'orchestratore main.py e aggiornato Step.md
</commit_message>
<xml_diff>
--- a/PMS_Report_DPR-385_Period_2024-01-01_to_2024-12-31.xlsx
+++ b/PMS_Report_DPR-385_Period_2024-01-01_to_2024-12-31.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Period 2024-01-01 to 2024-12-31</t>
+          <t>2024-01-01 to 2024-12-31</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-07-26 16:43</t>
+          <t>2026-07-26 16:46</t>
         </is>
       </c>
     </row>

</xml_diff>